<commit_message>
fix(entry): team import silently dropped teams with no Club or Seeding
readWorkbook trims trailing blank cells (Go GetRows parity), so an entries
row for a team with neither Club nor Seeding arrives as length 2 and the
row.length < 3 guard skipped it — e.g. Hemen, Ipad, and Hougang Green
vanished from Mens Team.xlsx. Skip only rows without a team name and treat
Club/Seeding/DOB/Gender as optional via nullish access.

Also relaxes the players-sheet guard the same way and refreshes the
Mens Team.xlsx fixture to the current 15-team file with regenerated
team goldens (deliberate divergence from the frozen Go baseline, which
had the same dropping behavior).
</commit_message>
<xml_diff>
--- a/web/testdata/Mens Team.xlsx
+++ b/web/testdata/Mens Team.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="14360" firstSheet="2" activeTab="1"/>
+    <workbookView windowHeight="14180" firstSheet="2"/>
   </bookViews>
   <sheets>
     <sheet name="entries" sheetId="3" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="73">
   <si>
     <t>SN</t>
   </si>
@@ -78,6 +78,30 @@
     <t>Ipad</t>
   </si>
   <si>
+    <t>Supamen</t>
+  </si>
+  <si>
+    <t>SGP</t>
+  </si>
+  <si>
+    <t>Sunsports</t>
+  </si>
+  <si>
+    <t>Chinese Swimming Club</t>
+  </si>
+  <si>
+    <t>Hougang Green</t>
+  </si>
+  <si>
+    <t>KSports</t>
+  </si>
+  <si>
+    <t>INA</t>
+  </si>
+  <si>
+    <t>Batam King</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
@@ -169,6 +193,60 @@
   </si>
   <si>
     <t>Izzac Quek</t>
+  </si>
+  <si>
+    <t>Poppy Tan</t>
+  </si>
+  <si>
+    <t>Lucy Chen</t>
+  </si>
+  <si>
+    <t>Wali Wali</t>
+  </si>
+  <si>
+    <t>Ghanah Nom</t>
+  </si>
+  <si>
+    <t>Peachy Tarisha</t>
+  </si>
+  <si>
+    <t>Albert</t>
+  </si>
+  <si>
+    <t>Einsteint</t>
+  </si>
+  <si>
+    <t>Sin Sin</t>
+  </si>
+  <si>
+    <t>Petr Pop</t>
+  </si>
+  <si>
+    <t>Gaji Guji</t>
+  </si>
+  <si>
+    <t>Elsa</t>
+  </si>
+  <si>
+    <t>Anna</t>
+  </si>
+  <si>
+    <t>Dogman</t>
+  </si>
+  <si>
+    <t>Doraemon</t>
+  </si>
+  <si>
+    <t>Anpori</t>
+  </si>
+  <si>
+    <t>Huliman</t>
+  </si>
+  <si>
+    <t>Quenti Loh</t>
+  </si>
+  <si>
+    <t>Pang Hu Shi</t>
   </si>
 </sst>
 </file>
@@ -1328,7 +1406,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1449,6 +1527,69 @@
         <v>15</v>
       </c>
     </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1458,7 +1599,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -1474,13 +1615,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -1491,13 +1632,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C2" s="2">
         <v>36893</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>4</v>
@@ -1508,13 +1649,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C3" s="2">
         <v>36894</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>4</v>
@@ -1525,13 +1666,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2">
         <v>36895</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>4</v>
@@ -1542,13 +1683,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2">
         <v>36896</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>6</v>
@@ -1559,13 +1700,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2">
         <v>36897</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>6</v>
@@ -1576,13 +1717,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C7" s="2">
         <v>36898</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>6</v>
@@ -1593,13 +1734,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2">
         <v>36899</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>7</v>
@@ -1610,13 +1751,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2">
         <v>36900</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>7</v>
@@ -1627,13 +1768,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C10" s="2">
         <v>36901</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>7</v>
@@ -1644,13 +1785,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C11" s="2">
         <v>36902</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
@@ -1661,13 +1802,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C12" s="2">
         <v>36903</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>8</v>
@@ -1678,13 +1819,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C13" s="2">
         <v>36904</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>8</v>
@@ -1695,13 +1836,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C14" s="2">
         <v>36905</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>9</v>
@@ -1712,13 +1853,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C15" s="2">
         <v>36906</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>9</v>
@@ -1729,13 +1870,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C16" s="2">
         <v>36907</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>9</v>
@@ -1746,13 +1887,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C17" s="2">
         <v>36908</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>11</v>
@@ -1763,13 +1904,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C18" s="2">
         <v>36909</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>11</v>
@@ -1780,13 +1921,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C19" s="2">
         <v>36910</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>11</v>
@@ -1797,13 +1938,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C20" s="2">
         <v>36911</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>12</v>
@@ -1814,13 +1955,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C21" s="2">
         <v>36912</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>12</v>
@@ -1831,13 +1972,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C22" s="2">
         <v>36913</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>12</v>
@@ -1848,13 +1989,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C23" s="2">
         <v>36914</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>14</v>
@@ -1865,13 +2006,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C24" s="2">
         <v>36915</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>14</v>
@@ -1882,13 +2023,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C25" s="2">
         <v>36916</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>14</v>
@@ -1899,13 +2040,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C26" s="2">
         <v>36917</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>15</v>
@@ -1916,13 +2057,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C27" s="2">
         <v>36918</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>15</v>
@@ -1933,16 +2074,322 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C28" s="2">
         <v>36919</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="2">
+        <v>36920</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="2">
+        <v>36921</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="2">
+        <v>36922</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" s="2">
+        <v>36923</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="2">
+        <v>36924</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="2">
+        <v>36925</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="2">
+        <v>36926</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="2">
+        <v>36927</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" s="2">
+        <v>36928</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C38" s="2">
+        <v>36929</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="2">
+        <v>36930</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="2">
+        <v>36931</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" s="2">
+        <v>36932</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C42" s="2">
+        <v>36933</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C43" s="2">
+        <v>36934</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C44" s="2">
+        <v>36935</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45" s="2">
+        <v>36936</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C46" s="2">
+        <v>36937</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>